<commit_message>
Ran All Benign NonIID
</commit_message>
<xml_diff>
--- a/Results.xlsx
+++ b/Results.xlsx
@@ -599,6 +599,9 @@
       <c r="I5" t="n">
         <v>0.1466666666666667</v>
       </c>
+      <c r="J5" t="n">
+        <v>0.084325</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
@@ -622,6 +625,9 @@
       <c r="I6" t="n">
         <v>0.18</v>
       </c>
+      <c r="J6" t="n">
+        <v>0.2527071428571429</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
@@ -645,6 +651,9 @@
       <c r="I7" t="n">
         <v>0.3585714285714285</v>
       </c>
+      <c r="J7" t="n">
+        <v>0.2572611111111111</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
@@ -668,6 +677,9 @@
       <c r="I8" t="n">
         <v>0.4255555555555556</v>
       </c>
+      <c r="J8" t="n">
+        <v>0.3903916666666667</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
@@ -691,6 +703,9 @@
       <c r="I9" t="n">
         <v>0.49</v>
       </c>
+      <c r="J9" t="n">
+        <v>0.4041571428571428</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
@@ -714,6 +729,9 @@
       <c r="I10" t="n">
         <v>0.456</v>
       </c>
+      <c r="J10" t="n">
+        <v>0.509775</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
@@ -737,6 +755,9 @@
       <c r="I11" t="n">
         <v>0.512</v>
       </c>
+      <c r="J11" t="n">
+        <v>0.5659884615384616</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
@@ -760,6 +781,9 @@
       <c r="I12" t="n">
         <v>0.4925</v>
       </c>
+      <c r="J12" t="n">
+        <v>0.6995205882352941</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
@@ -783,6 +807,9 @@
       <c r="I13" t="n">
         <v>0.5328571428571428</v>
       </c>
+      <c r="J13" t="n">
+        <v>0.646334375</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
@@ -806,6 +833,9 @@
       <c r="I14" t="n">
         <v>0.5477777777777777</v>
       </c>
+      <c r="J14" t="n">
+        <v>0.7051977272727273</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -829,6 +859,9 @@
       <c r="I15" t="n">
         <v>0.5416666666666666</v>
       </c>
+      <c r="J15" t="n">
+        <v>0.7101333333333334</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
@@ -852,6 +885,9 @@
       <c r="I16" t="n">
         <v>0.5587500000000001</v>
       </c>
+      <c r="J16" t="n">
+        <v>0.7276179487179487</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
@@ -875,6 +911,9 @@
       <c r="I17" t="n">
         <v>0.58</v>
       </c>
+      <c r="J17" t="n">
+        <v>0.7821196078431373</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
@@ -898,6 +937,9 @@
       <c r="I18" t="n">
         <v>0.5718181818181818</v>
       </c>
+      <c r="J18" t="n">
+        <v>0.8010444444444444</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
@@ -921,6 +963,9 @@
       <c r="I19" t="n">
         <v>0.5685714285714285</v>
       </c>
+      <c r="J19" t="n">
+        <v>0.777974358974359</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
@@ -944,6 +989,9 @@
       <c r="I20" t="n">
         <v>0.57875</v>
       </c>
+      <c r="J20" t="n">
+        <v>0.674482</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
@@ -967,6 +1015,9 @@
       <c r="I21" t="n">
         <v>0.5875</v>
       </c>
+      <c r="J21" t="n">
+        <v>0.6924926829268293</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
@@ -990,6 +1041,9 @@
       <c r="I22" t="n">
         <v>0.5639999999999999</v>
       </c>
+      <c r="J22" t="n">
+        <v>0.786239393939394</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
@@ -1013,6 +1067,9 @@
       <c r="I23" t="n">
         <v>0.5909090909090909</v>
       </c>
+      <c r="J23" t="n">
+        <v>0.8290617647058824</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
@@ -1036,6 +1093,9 @@
       <c r="I24" t="n">
         <v>0.5911111111111111</v>
       </c>
+      <c r="J24" t="n">
+        <v>0.7833928571428571</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
@@ -1059,6 +1119,9 @@
       <c r="I25" t="n">
         <v>0.595</v>
       </c>
+      <c r="J25" t="n">
+        <v>0.7791833333333333</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
@@ -1082,6 +1145,9 @@
       <c r="I26" t="n">
         <v>0.5988888888888889</v>
       </c>
+      <c r="J26" t="n">
+        <v>0.8023947368421053</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
@@ -1105,6 +1171,9 @@
       <c r="I27" t="n">
         <v>0.5544444444444445</v>
       </c>
+      <c r="J27" t="n">
+        <v>0.794712</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
@@ -1128,6 +1197,9 @@
       <c r="I28" t="n">
         <v>0.59</v>
       </c>
+      <c r="J28" t="n">
+        <v>0.8642666666666668</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
@@ -1151,6 +1223,9 @@
       <c r="I29" t="n">
         <v>0.5972727272727272</v>
       </c>
+      <c r="J29" t="n">
+        <v>0.8025583333333333</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
@@ -1174,6 +1249,9 @@
       <c r="I30" t="n">
         <v>0.5999999999999999</v>
       </c>
+      <c r="J30" t="n">
+        <v>0.841264864864865</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
@@ -1197,6 +1275,9 @@
       <c r="I31" t="n">
         <v>0.5924999999999999</v>
       </c>
+      <c r="J31" t="n">
+        <v>0.8277212121212121</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
@@ -1220,6 +1301,9 @@
       <c r="I32" t="n">
         <v>0.58</v>
       </c>
+      <c r="J32" t="n">
+        <v>0.8714515151515152</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
@@ -1243,6 +1327,9 @@
       <c r="I33" t="n">
         <v>0.6259999999999999</v>
       </c>
+      <c r="J33" t="n">
+        <v>0.8257514285714286</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
@@ -1266,6 +1353,9 @@
       <c r="I34" t="n">
         <v>0.594</v>
       </c>
+      <c r="J34" t="n">
+        <v>0.713465</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
@@ -1289,6 +1379,9 @@
       <c r="I35" t="n">
         <v>0.601</v>
       </c>
+      <c r="J35" t="n">
+        <v>0.8098421052631579</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
@@ -1312,6 +1405,9 @@
       <c r="I36" t="n">
         <v>0.5766666666666668</v>
       </c>
+      <c r="J36" t="n">
+        <v>0.8045666666666667</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
@@ -1335,6 +1431,9 @@
       <c r="I37" t="n">
         <v>0.6174999999999999</v>
       </c>
+      <c r="J37" t="n">
+        <v>0.7566081081081082</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
@@ -1358,6 +1457,9 @@
       <c r="I38" t="n">
         <v>0.5955555555555555</v>
       </c>
+      <c r="J38" t="n">
+        <v>0.8094117647058825</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
@@ -1381,6 +1483,9 @@
       <c r="I39" t="n">
         <v>0.592</v>
       </c>
+      <c r="J39" t="n">
+        <v>0.857563043478261</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
@@ -1404,6 +1509,9 @@
       <c r="I40" t="n">
         <v>0.5787500000000001</v>
       </c>
+      <c r="J40" t="n">
+        <v>0.8153321428571428</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
@@ -1427,6 +1535,9 @@
       <c r="I41" t="n">
         <v>0.5912499999999999</v>
       </c>
+      <c r="J41" t="n">
+        <v>0.83691875</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
@@ -1450,6 +1561,9 @@
       <c r="I42" t="n">
         <v>0.6022222222222222</v>
       </c>
+      <c r="J42" t="n">
+        <v>0.8283978260869567</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
@@ -1473,6 +1587,9 @@
       <c r="I43" t="n">
         <v>0.611</v>
       </c>
+      <c r="J43" t="n">
+        <v>0.8282827586206897</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
@@ -1496,6 +1613,9 @@
       <c r="I44" t="n">
         <v>0.6190000000000001</v>
       </c>
+      <c r="J44" t="n">
+        <v>0.8807318181818182</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
@@ -1519,6 +1639,9 @@
       <c r="I45" t="n">
         <v>0.60625</v>
       </c>
+      <c r="J45" t="n">
+        <v>0.8044952380952382</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
@@ -1542,6 +1665,9 @@
       <c r="I46" t="n">
         <v>0.6259999999999999</v>
       </c>
+      <c r="J46" t="n">
+        <v>0.8225977777777778</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
@@ -1565,6 +1691,9 @@
       <c r="I47" t="n">
         <v>0.6299999999999999</v>
       </c>
+      <c r="J47" t="n">
+        <v>0.8230216216216216</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
@@ -1588,6 +1717,9 @@
       <c r="I48" t="n">
         <v>0.6512499999999999</v>
       </c>
+      <c r="J48" t="n">
+        <v>0.8747666666666668</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
@@ -1611,6 +1743,9 @@
       <c r="I49" t="n">
         <v>0.616</v>
       </c>
+      <c r="J49" t="n">
+        <v>0.8695774193548389</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
@@ -1634,6 +1769,9 @@
       <c r="I50" t="n">
         <v>0.633</v>
       </c>
+      <c r="J50" t="n">
+        <v>0.8196439024390245</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
@@ -1657,6 +1795,9 @@
       <c r="I51" t="n">
         <v>0.6511111111111111</v>
       </c>
+      <c r="J51" t="n">
+        <v>0.8887681818181818</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
@@ -1680,6 +1821,9 @@
       <c r="I52" t="n">
         <v>0.621</v>
       </c>
+      <c r="J52" t="n">
+        <v>0.8855155555555555</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
@@ -1703,6 +1847,9 @@
       <c r="I53" t="n">
         <v>0.6425</v>
       </c>
+      <c r="J53" t="n">
+        <v>0.76078</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
@@ -1726,6 +1873,9 @@
       <c r="I54" t="n">
         <v>0.625</v>
       </c>
+      <c r="J54" t="n">
+        <v>0.8361736842105261</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
@@ -1749,6 +1899,9 @@
       <c r="I55" t="n">
         <v>0.60125</v>
       </c>
+      <c r="J55" t="n">
+        <v>0.8737023809523811</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
@@ -1772,6 +1925,9 @@
       <c r="I56" t="n">
         <v>0.62</v>
       </c>
+      <c r="J56" t="n">
+        <v>0.9107047619047619</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
@@ -1795,6 +1951,9 @@
       <c r="I57" t="n">
         <v>0.6377777777777778</v>
       </c>
+      <c r="J57" t="n">
+        <v>0.8687533333333335</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
@@ -1818,6 +1977,9 @@
       <c r="I58" t="n">
         <v>0.62</v>
       </c>
+      <c r="J58" t="n">
+        <v>0.842967857142857</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
@@ -1841,6 +2003,9 @@
       <c r="I59" t="n">
         <v>0.6437499999999999</v>
       </c>
+      <c r="J59" t="n">
+        <v>0.8244981132075472</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
@@ -1864,6 +2029,9 @@
       <c r="I60" t="n">
         <v>0.65</v>
       </c>
+      <c r="J60" t="n">
+        <v>0.8236529411764707</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
@@ -1887,6 +2055,9 @@
       <c r="I61" t="n">
         <v>0.6150000000000001</v>
       </c>
+      <c r="J61" t="n">
+        <v>0.8588763157894738</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
@@ -1910,6 +2081,9 @@
       <c r="I62" t="n">
         <v>0.6275000000000001</v>
       </c>
+      <c r="J62" t="n">
+        <v>0.8965612903225807</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
@@ -1933,6 +2107,9 @@
       <c r="I63" t="n">
         <v>0.6116666666666667</v>
       </c>
+      <c r="J63" t="n">
+        <v>0.8717281250000001</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
@@ -1956,6 +2133,9 @@
       <c r="I64" t="n">
         <v>0.6357142857142856</v>
       </c>
+      <c r="J64" t="n">
+        <v>0.8515315789473685</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
@@ -1979,6 +2159,9 @@
       <c r="I65" t="n">
         <v>0.6266666666666666</v>
       </c>
+      <c r="J65" t="n">
+        <v>0.8058722222222223</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">
@@ -2002,6 +2185,9 @@
       <c r="I66" t="n">
         <v>0.6233333333333333</v>
       </c>
+      <c r="J66" t="n">
+        <v>0.8136958333333334</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="n">
@@ -2025,6 +2211,9 @@
       <c r="I67" t="n">
         <v>0.6422222222222224</v>
       </c>
+      <c r="J67" t="n">
+        <v>0.8007903225806452</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="n">
@@ -2048,6 +2237,9 @@
       <c r="I68" t="n">
         <v>0.603</v>
       </c>
+      <c r="J68" t="n">
+        <v>0.8431424999999999</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="n">
@@ -2071,6 +2263,9 @@
       <c r="I69" t="n">
         <v>0.65</v>
       </c>
+      <c r="J69" t="n">
+        <v>0.8015155172413793</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="n">
@@ -2094,6 +2289,9 @@
       <c r="I70" t="n">
         <v>0.594</v>
       </c>
+      <c r="J70" t="n">
+        <v>0.8374625</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
@@ -2117,6 +2315,9 @@
       <c r="I71" t="n">
         <v>0.6033333333333333</v>
       </c>
+      <c r="J71" t="n">
+        <v>0.812629268292683</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="n">
@@ -2140,6 +2341,9 @@
       <c r="I72" t="n">
         <v>0.6224999999999999</v>
       </c>
+      <c r="J72" t="n">
+        <v>0.8550695652173913</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="n">
@@ -2163,6 +2367,9 @@
       <c r="I73" t="n">
         <v>0.626</v>
       </c>
+      <c r="J73" t="n">
+        <v>0.7988055555555555</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="n">
@@ -2186,6 +2393,9 @@
       <c r="I74" t="n">
         <v>0.61</v>
       </c>
+      <c r="J74" t="n">
+        <v>0.8802259259259259</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="n">
@@ -2209,6 +2419,9 @@
       <c r="I75" t="n">
         <v>0.6353846153846154</v>
       </c>
+      <c r="J75" t="n">
+        <v>0.8824487804878048</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="n">
@@ -2232,6 +2445,9 @@
       <c r="I76" t="n">
         <v>0.626</v>
       </c>
+      <c r="J76" t="n">
+        <v>0.8494771428571427</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="1" t="n">
@@ -2255,6 +2471,9 @@
       <c r="I77" t="n">
         <v>0.61</v>
       </c>
+      <c r="J77" t="n">
+        <v>0.8099722222222222</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="1" t="n">
@@ -2278,6 +2497,9 @@
       <c r="I78" t="n">
         <v>0.6024999999999999</v>
       </c>
+      <c r="J78" t="n">
+        <v>0.8352948717948717</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="1" t="n">
@@ -2301,6 +2523,9 @@
       <c r="I79" t="n">
         <v>0.6172727272727272</v>
       </c>
+      <c r="J79" t="n">
+        <v>0.7850076923076924</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="1" t="n">
@@ -2324,6 +2549,9 @@
       <c r="I80" t="n">
         <v>0.6323076923076923</v>
       </c>
+      <c r="J80" t="n">
+        <v>0.8836761904761905</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="1" t="n">
@@ -2347,6 +2575,9 @@
       <c r="I81" t="n">
         <v>0.6381818181818182</v>
       </c>
+      <c r="J81" t="n">
+        <v>0.7918697674418603</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="1" t="n">
@@ -2370,6 +2601,9 @@
       <c r="I82" t="n">
         <v>0.6300000000000001</v>
       </c>
+      <c r="J82" t="n">
+        <v>0.8031800000000001</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="1" t="n">
@@ -2393,6 +2627,9 @@
       <c r="I83" t="n">
         <v>0.6377777777777779</v>
       </c>
+      <c r="J83" t="n">
+        <v>0.8663222222222221</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="1" t="n">
@@ -2416,6 +2653,9 @@
       <c r="I84" t="n">
         <v>0.6077777777777779</v>
       </c>
+      <c r="J84" t="n">
+        <v>0.8505545454545456</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="1" t="n">
@@ -2439,6 +2679,9 @@
       <c r="I85" t="n">
         <v>0.6171428571428572</v>
       </c>
+      <c r="J85" t="n">
+        <v>0.8456575757575757</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="1" t="n">
@@ -2462,6 +2705,9 @@
       <c r="I86" t="n">
         <v>0.636</v>
       </c>
+      <c r="J86" t="n">
+        <v>0.8337040816326531</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="1" t="n">
@@ -2485,6 +2731,9 @@
       <c r="I87" t="n">
         <v>0.648</v>
       </c>
+      <c r="J87" t="n">
+        <v>0.8017185185185185</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="1" t="n">
@@ -2508,6 +2757,9 @@
       <c r="I88" t="n">
         <v>0.6388888888888888</v>
       </c>
+      <c r="J88" t="n">
+        <v>0.8196030303030303</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="1" t="n">
@@ -2531,6 +2783,9 @@
       <c r="I89" t="n">
         <v>0.6388888888888888</v>
       </c>
+      <c r="J89" t="n">
+        <v>0.8074947368421052</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="1" t="n">
@@ -2554,6 +2809,9 @@
       <c r="I90" t="n">
         <v>0.6111111111111112</v>
       </c>
+      <c r="J90" t="n">
+        <v>0.781253125</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="1" t="n">
@@ -2577,6 +2835,9 @@
       <c r="I91" t="n">
         <v>0.63</v>
       </c>
+      <c r="J91" t="n">
+        <v>0.8277413793103449</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="1" t="n">
@@ -2600,6 +2861,9 @@
       <c r="I92" t="n">
         <v>0.632</v>
       </c>
+      <c r="J92" t="n">
+        <v>0.8489088888888888</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="1" t="n">
@@ -2623,6 +2887,9 @@
       <c r="I93" t="n">
         <v>0.6325000000000001</v>
       </c>
+      <c r="J93" t="n">
+        <v>0.8572111111111111</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="1" t="n">
@@ -2646,6 +2913,9 @@
       <c r="I94" t="n">
         <v>0.6055555555555556</v>
       </c>
+      <c r="J94" t="n">
+        <v>0.7635352941176471</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="n">
@@ -2669,6 +2939,9 @@
       <c r="I95" t="n">
         <v>0.6</v>
       </c>
+      <c r="J95" t="n">
+        <v>0.8265319999999999</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="1" t="n">
@@ -2692,6 +2965,9 @@
       <c r="I96" t="n">
         <v>0.623</v>
       </c>
+      <c r="J96" t="n">
+        <v>0.8006685714285714</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="1" t="n">
@@ -2715,6 +2991,9 @@
       <c r="I97" t="n">
         <v>0.6466666666666666</v>
       </c>
+      <c r="J97" t="n">
+        <v>0.7916</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="1" t="n">
@@ -2738,6 +3017,9 @@
       <c r="I98" t="n">
         <v>0.675</v>
       </c>
+      <c r="J98" t="n">
+        <v>0.8065529411764706</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="1" t="n">
@@ -2761,6 +3043,9 @@
       <c r="I99" t="n">
         <v>0.65</v>
       </c>
+      <c r="J99" t="n">
+        <v>0.8485624999999999</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="1" t="n">
@@ -2784,6 +3069,9 @@
       <c r="I100" t="n">
         <v>0.6011111111111112</v>
       </c>
+      <c r="J100" t="n">
+        <v>0.8383518518518519</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="1" t="n">
@@ -2807,6 +3095,9 @@
       <c r="I101" t="n">
         <v>0.6466666666666667</v>
       </c>
+      <c r="J101" t="n">
+        <v>0.8121136363636364</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="1" t="n">
@@ -2830,6 +3121,9 @@
       <c r="I102" t="n">
         <v>0.634</v>
       </c>
+      <c r="J102" t="n">
+        <v>0.8871957446808511</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="1" t="n">
@@ -2853,6 +3147,9 @@
       <c r="I103" t="n">
         <v>0.6377777777777778</v>
       </c>
+      <c r="J103" t="n">
+        <v>0.8266685714285714</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="1" t="n">
@@ -2875,6 +3172,9 @@
       </c>
       <c r="I104" t="n">
         <v>0.6518181818181819</v>
+      </c>
+      <c r="J104" t="n">
+        <v>0.8704032258064517</v>
       </c>
     </row>
     <row r="106">
@@ -2923,6 +3223,9 @@
       <c r="I108" t="n">
         <v>1</v>
       </c>
+      <c r="J108" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="1" t="n">
@@ -2946,6 +3249,9 @@
       <c r="I109" t="n">
         <v>1</v>
       </c>
+      <c r="J109" t="n">
+        <v>0.7692307692307693</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="1" t="n">
@@ -2969,6 +3275,9 @@
       <c r="I110" t="n">
         <v>1</v>
       </c>
+      <c r="J110" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="1" t="n">
@@ -2992,6 +3301,9 @@
       <c r="I111" t="n">
         <v>1</v>
       </c>
+      <c r="J111" t="n">
+        <v>0.75</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="1" t="n">
@@ -3015,6 +3327,9 @@
       <c r="I112" t="n">
         <v>1</v>
       </c>
+      <c r="J112" t="n">
+        <v>0.8571428571428571</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="1" t="n">
@@ -3038,6 +3353,9 @@
       <c r="I113" t="n">
         <v>1</v>
       </c>
+      <c r="J113" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="1" t="n">
@@ -3061,6 +3379,9 @@
       <c r="I114" t="n">
         <v>1</v>
       </c>
+      <c r="J114" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="1" t="n">
@@ -3084,6 +3405,9 @@
       <c r="I115" t="n">
         <v>1</v>
       </c>
+      <c r="J115" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="1" t="n">
@@ -3107,6 +3431,9 @@
       <c r="I116" t="n">
         <v>1</v>
       </c>
+      <c r="J116" t="n">
+        <v>0.8333333333333334</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="1" t="n">
@@ -3130,6 +3457,9 @@
       <c r="I117" t="n">
         <v>1</v>
       </c>
+      <c r="J117" t="n">
+        <v>0.8571428571428571</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="1" t="n">
@@ -3153,6 +3483,9 @@
       <c r="I118" t="n">
         <v>1</v>
       </c>
+      <c r="J118" t="n">
+        <v>0.8333333333333334</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="n">
@@ -3176,6 +3509,9 @@
       <c r="I119" t="n">
         <v>1</v>
       </c>
+      <c r="J119" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="1" t="n">
@@ -3199,6 +3535,9 @@
       <c r="I120" t="n">
         <v>1</v>
       </c>
+      <c r="J120" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="n">
@@ -3222,6 +3561,9 @@
       <c r="I121" t="n">
         <v>1</v>
       </c>
+      <c r="J121" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="n">
@@ -3245,6 +3587,9 @@
       <c r="I122" t="n">
         <v>1</v>
       </c>
+      <c r="J122" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="n">
@@ -3268,6 +3613,9 @@
       <c r="I123" t="n">
         <v>1</v>
       </c>
+      <c r="J123" t="n">
+        <v>0.3333333333333333</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="n">
@@ -3291,6 +3639,9 @@
       <c r="I124" t="n">
         <v>1</v>
       </c>
+      <c r="J124" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="1" t="n">
@@ -3314,6 +3665,9 @@
       <c r="I125" t="n">
         <v>1</v>
       </c>
+      <c r="J125" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="1" t="n">
@@ -3337,6 +3691,9 @@
       <c r="I126" t="n">
         <v>1</v>
       </c>
+      <c r="J126" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="n">
@@ -3360,6 +3717,9 @@
       <c r="I127" t="n">
         <v>1</v>
       </c>
+      <c r="J127" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="1" t="n">
@@ -3383,6 +3743,9 @@
       <c r="I128" t="n">
         <v>1</v>
       </c>
+      <c r="J128" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="1" t="n">
@@ -3406,6 +3769,9 @@
       <c r="I129" t="n">
         <v>1</v>
       </c>
+      <c r="J129" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="1" t="n">
@@ -3429,6 +3795,9 @@
       <c r="I130" t="n">
         <v>1</v>
       </c>
+      <c r="J130" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="1" t="n">
@@ -3452,6 +3821,9 @@
       <c r="I131" t="n">
         <v>1</v>
       </c>
+      <c r="J131" t="n">
+        <v>0.8571428571428571</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="1" t="n">
@@ -3475,6 +3847,9 @@
       <c r="I132" t="n">
         <v>1</v>
       </c>
+      <c r="J132" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="1" t="n">
@@ -3498,6 +3873,9 @@
       <c r="I133" t="n">
         <v>1</v>
       </c>
+      <c r="J133" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="1" t="n">
@@ -3521,6 +3899,9 @@
       <c r="I134" t="n">
         <v>1</v>
       </c>
+      <c r="J134" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="1" t="n">
@@ -3544,6 +3925,9 @@
       <c r="I135" t="n">
         <v>1</v>
       </c>
+      <c r="J135" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="1" t="n">
@@ -3567,6 +3951,9 @@
       <c r="I136" t="n">
         <v>1</v>
       </c>
+      <c r="J136" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="n">
@@ -3590,6 +3977,9 @@
       <c r="I137" t="n">
         <v>1</v>
       </c>
+      <c r="J137" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="n">
@@ -3613,6 +4003,9 @@
       <c r="I138" t="n">
         <v>1</v>
       </c>
+      <c r="J138" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="n">
@@ -3636,6 +4029,9 @@
       <c r="I139" t="n">
         <v>1</v>
       </c>
+      <c r="J139" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="n">
@@ -3659,6 +4055,9 @@
       <c r="I140" t="n">
         <v>1</v>
       </c>
+      <c r="J140" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="1" t="n">
@@ -3682,6 +4081,9 @@
       <c r="I141" t="n">
         <v>1</v>
       </c>
+      <c r="J141" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="1" t="n">
@@ -3705,6 +4107,9 @@
       <c r="I142" t="n">
         <v>1</v>
       </c>
+      <c r="J142" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="1" t="n">
@@ -3728,6 +4133,9 @@
       <c r="I143" t="n">
         <v>1</v>
       </c>
+      <c r="J143" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="1" t="n">
@@ -3751,6 +4159,9 @@
       <c r="I144" t="n">
         <v>1</v>
       </c>
+      <c r="J144" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="1" t="n">
@@ -3774,6 +4185,9 @@
       <c r="I145" t="n">
         <v>1</v>
       </c>
+      <c r="J145" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="n">
@@ -3797,6 +4211,9 @@
       <c r="I146" t="n">
         <v>1</v>
       </c>
+      <c r="J146" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="n">
@@ -3820,6 +4237,9 @@
       <c r="I147" t="n">
         <v>1</v>
       </c>
+      <c r="J147" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="n">
@@ -3843,6 +4263,9 @@
       <c r="I148" t="n">
         <v>1</v>
       </c>
+      <c r="J148" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="n">
@@ -3866,6 +4289,9 @@
       <c r="I149" t="n">
         <v>1</v>
       </c>
+      <c r="J149" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="n">
@@ -3889,6 +4315,9 @@
       <c r="I150" t="n">
         <v>1</v>
       </c>
+      <c r="J150" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="n">
@@ -3912,6 +4341,9 @@
       <c r="I151" t="n">
         <v>1</v>
       </c>
+      <c r="J151" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="n">
@@ -3935,6 +4367,9 @@
       <c r="I152" t="n">
         <v>1</v>
       </c>
+      <c r="J152" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="n">
@@ -3958,6 +4393,9 @@
       <c r="I153" t="n">
         <v>1</v>
       </c>
+      <c r="J153" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="n">
@@ -3981,6 +4419,9 @@
       <c r="I154" t="n">
         <v>1</v>
       </c>
+      <c r="J154" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="n">
@@ -4004,6 +4445,9 @@
       <c r="I155" t="n">
         <v>1</v>
       </c>
+      <c r="J155" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="n">
@@ -4027,6 +4471,9 @@
       <c r="I156" t="n">
         <v>1</v>
       </c>
+      <c r="J156" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="n">
@@ -4050,6 +4497,9 @@
       <c r="I157" t="n">
         <v>1</v>
       </c>
+      <c r="J157" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="n">
@@ -4073,6 +4523,9 @@
       <c r="I158" t="n">
         <v>1</v>
       </c>
+      <c r="J158" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="n">
@@ -4096,6 +4549,9 @@
       <c r="I159" t="n">
         <v>1</v>
       </c>
+      <c r="J159" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="1" t="n">
@@ -4119,6 +4575,9 @@
       <c r="I160" t="n">
         <v>1</v>
       </c>
+      <c r="J160" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="n">
@@ -4142,6 +4601,9 @@
       <c r="I161" t="n">
         <v>1</v>
       </c>
+      <c r="J161" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="n">
@@ -4165,6 +4627,9 @@
       <c r="I162" t="n">
         <v>1</v>
       </c>
+      <c r="J162" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="1" t="n">
@@ -4188,6 +4653,9 @@
       <c r="I163" t="n">
         <v>1</v>
       </c>
+      <c r="J163" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="1" t="n">
@@ -4211,6 +4679,9 @@
       <c r="I164" t="n">
         <v>1</v>
       </c>
+      <c r="J164" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="1" t="n">
@@ -4234,6 +4705,9 @@
       <c r="I165" t="n">
         <v>1</v>
       </c>
+      <c r="J165" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="1" t="n">
@@ -4257,6 +4731,9 @@
       <c r="I166" t="n">
         <v>1</v>
       </c>
+      <c r="J166" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="1" t="n">
@@ -4280,6 +4757,9 @@
       <c r="I167" t="n">
         <v>1</v>
       </c>
+      <c r="J167" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="1" t="n">
@@ -4303,6 +4783,9 @@
       <c r="I168" t="n">
         <v>1</v>
       </c>
+      <c r="J168" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="1" t="n">
@@ -4326,6 +4809,9 @@
       <c r="I169" t="n">
         <v>1</v>
       </c>
+      <c r="J169" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="1" t="n">
@@ -4349,6 +4835,9 @@
       <c r="I170" t="n">
         <v>1</v>
       </c>
+      <c r="J170" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="1" t="n">
@@ -4372,6 +4861,9 @@
       <c r="I171" t="n">
         <v>1</v>
       </c>
+      <c r="J171" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="1" t="n">
@@ -4395,6 +4887,9 @@
       <c r="I172" t="n">
         <v>1</v>
       </c>
+      <c r="J172" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="1" t="n">
@@ -4418,6 +4913,9 @@
       <c r="I173" t="n">
         <v>1</v>
       </c>
+      <c r="J173" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="1" t="n">
@@ -4441,6 +4939,9 @@
       <c r="I174" t="n">
         <v>1</v>
       </c>
+      <c r="J174" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="1" t="n">
@@ -4464,6 +4965,9 @@
       <c r="I175" t="n">
         <v>1</v>
       </c>
+      <c r="J175" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="1" t="n">
@@ -4487,6 +4991,9 @@
       <c r="I176" t="n">
         <v>1</v>
       </c>
+      <c r="J176" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="1" t="n">
@@ -4510,6 +5017,9 @@
       <c r="I177" t="n">
         <v>1</v>
       </c>
+      <c r="J177" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="1" t="n">
@@ -4533,6 +5043,9 @@
       <c r="I178" t="n">
         <v>1</v>
       </c>
+      <c r="J178" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="1" t="n">
@@ -4556,6 +5069,9 @@
       <c r="I179" t="n">
         <v>1</v>
       </c>
+      <c r="J179" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="1" t="n">
@@ -4579,6 +5095,9 @@
       <c r="I180" t="n">
         <v>1</v>
       </c>
+      <c r="J180" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="1" t="n">
@@ -4602,6 +5121,9 @@
       <c r="I181" t="n">
         <v>1</v>
       </c>
+      <c r="J181" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="1" t="n">
@@ -4625,6 +5147,9 @@
       <c r="I182" t="n">
         <v>1</v>
       </c>
+      <c r="J182" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="1" t="n">
@@ -4648,6 +5173,9 @@
       <c r="I183" t="n">
         <v>1</v>
       </c>
+      <c r="J183" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="1" t="n">
@@ -4671,6 +5199,9 @@
       <c r="I184" t="n">
         <v>1</v>
       </c>
+      <c r="J184" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="1" t="n">
@@ -4694,6 +5225,9 @@
       <c r="I185" t="n">
         <v>1</v>
       </c>
+      <c r="J185" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="1" t="n">
@@ -4717,6 +5251,9 @@
       <c r="I186" t="n">
         <v>1</v>
       </c>
+      <c r="J186" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="1" t="n">
@@ -4740,6 +5277,9 @@
       <c r="I187" t="n">
         <v>1</v>
       </c>
+      <c r="J187" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="1" t="n">
@@ -4763,6 +5303,9 @@
       <c r="I188" t="n">
         <v>1</v>
       </c>
+      <c r="J188" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="1" t="n">
@@ -4786,6 +5329,9 @@
       <c r="I189" t="n">
         <v>1</v>
       </c>
+      <c r="J189" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="1" t="n">
@@ -4809,6 +5355,9 @@
       <c r="I190" t="n">
         <v>1</v>
       </c>
+      <c r="J190" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="1" t="n">
@@ -4832,6 +5381,9 @@
       <c r="I191" t="n">
         <v>1</v>
       </c>
+      <c r="J191" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="1" t="n">
@@ -4855,6 +5407,9 @@
       <c r="I192" t="n">
         <v>1</v>
       </c>
+      <c r="J192" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="1" t="n">
@@ -4878,6 +5433,9 @@
       <c r="I193" t="n">
         <v>1</v>
       </c>
+      <c r="J193" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="1" t="n">
@@ -4901,6 +5459,9 @@
       <c r="I194" t="n">
         <v>1</v>
       </c>
+      <c r="J194" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="1" t="n">
@@ -4924,6 +5485,9 @@
       <c r="I195" t="n">
         <v>1</v>
       </c>
+      <c r="J195" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="1" t="n">
@@ -4947,6 +5511,9 @@
       <c r="I196" t="n">
         <v>1</v>
       </c>
+      <c r="J196" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="1" t="n">
@@ -4970,6 +5537,9 @@
       <c r="I197" t="n">
         <v>1</v>
       </c>
+      <c r="J197" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="1" t="n">
@@ -4993,6 +5563,9 @@
       <c r="I198" t="n">
         <v>1</v>
       </c>
+      <c r="J198" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="1" t="n">
@@ -5016,6 +5589,9 @@
       <c r="I199" t="n">
         <v>1</v>
       </c>
+      <c r="J199" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="1" t="n">
@@ -5039,6 +5615,9 @@
       <c r="I200" t="n">
         <v>1</v>
       </c>
+      <c r="J200" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="1" t="n">
@@ -5062,6 +5641,9 @@
       <c r="I201" t="n">
         <v>1</v>
       </c>
+      <c r="J201" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="1" t="n">
@@ -5085,6 +5667,9 @@
       <c r="I202" t="n">
         <v>1</v>
       </c>
+      <c r="J202" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="1" t="n">
@@ -5108,6 +5693,9 @@
       <c r="I203" t="n">
         <v>1</v>
       </c>
+      <c r="J203" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="1" t="n">
@@ -5131,6 +5719,9 @@
       <c r="I204" t="n">
         <v>1</v>
       </c>
+      <c r="J204" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="1" t="n">
@@ -5154,6 +5745,9 @@
       <c r="I205" t="n">
         <v>1</v>
       </c>
+      <c r="J205" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="1" t="n">
@@ -5177,6 +5771,9 @@
       <c r="I206" t="n">
         <v>1</v>
       </c>
+      <c r="J206" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="1" t="n">
@@ -5198,6 +5795,9 @@
         <v>100</v>
       </c>
       <c r="I207" t="n">
+        <v>1</v>
+      </c>
+      <c r="J207" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5247,6 +5847,9 @@
       <c r="I212" t="n">
         <v>0.00765</v>
       </c>
+      <c r="J212" t="n">
+        <v>0.8452</v>
+      </c>
     </row>
     <row r="213">
       <c r="A213" s="1" t="n">
@@ -5270,6 +5873,9 @@
       <c r="I213" t="n">
         <v>0.006675</v>
       </c>
+      <c r="J213" t="n">
+        <v>0.6774625000000001</v>
+      </c>
     </row>
     <row r="214">
       <c r="A214" s="1" t="n">
@@ -5293,6 +5899,9 @@
       <c r="I214" t="n">
         <v>0.0070375</v>
       </c>
+      <c r="J214" t="n">
+        <v>0.7674111111111112</v>
+      </c>
     </row>
     <row r="215">
       <c r="A215" s="1" t="n">
@@ -5316,6 +5925,9 @@
       <c r="I215" t="n">
         <v>0.009049999999999999</v>
       </c>
+      <c r="J215" t="n">
+        <v>0.7663500000000001</v>
+      </c>
     </row>
     <row r="216">
       <c r="A216" s="1" t="n">
@@ -5339,6 +5951,9 @@
       <c r="I216" t="n">
         <v>0.007285714285714286</v>
       </c>
+      <c r="J216" t="n">
+        <v>0.6505777777777778</v>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="1" t="n">
@@ -5362,6 +5977,9 @@
       <c r="I217" t="n">
         <v>0.006057142857142857</v>
       </c>
+      <c r="J217" t="n">
+        <v>0.6559818181818181</v>
+      </c>
     </row>
     <row r="218">
       <c r="A218" s="1" t="n">
@@ -5385,6 +6003,9 @@
       <c r="I218" t="n">
         <v>0.01086</v>
       </c>
+      <c r="J218" t="n">
+        <v>0.4963333333333333</v>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="1" t="n">
@@ -5408,6 +6029,9 @@
       <c r="I219" t="n">
         <v>0.0125</v>
       </c>
+      <c r="J219" t="n">
+        <v>0.5920555555555556</v>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="1" t="n">
@@ -5431,6 +6055,9 @@
       <c r="I220" t="n">
         <v>0.00925</v>
       </c>
+      <c r="J220" t="n">
+        <v>0.5877</v>
+      </c>
     </row>
     <row r="221">
       <c r="A221" s="1" t="n">
@@ -5454,6 +6081,9 @@
       <c r="I221" t="n">
         <v>0.0123625</v>
       </c>
+      <c r="J221" t="n">
+        <v>0.7752444444444444</v>
+      </c>
     </row>
     <row r="222">
       <c r="A222" s="1" t="n">
@@ -5477,6 +6107,9 @@
       <c r="I222" t="n">
         <v>0.010725</v>
       </c>
+      <c r="J222" t="n">
+        <v>0.64361</v>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="1" t="n">
@@ -5500,6 +6133,9 @@
       <c r="I223" t="n">
         <v>0.01165714285714286</v>
       </c>
+      <c r="J223" t="n">
+        <v>0.4885714285714285</v>
+      </c>
     </row>
     <row r="224">
       <c r="A224" s="1" t="n">
@@ -5523,6 +6159,9 @@
       <c r="I224" t="n">
         <v>0.009600000000000001</v>
       </c>
+      <c r="J224" t="n">
+        <v>0.6527000000000001</v>
+      </c>
     </row>
     <row r="225">
       <c r="A225" s="1" t="n">
@@ -5546,6 +6185,9 @@
       <c r="I225" t="n">
         <v>0.008685714285714286</v>
       </c>
+      <c r="J225" t="n">
+        <v>0.5255399999999999</v>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="1" t="n">
@@ -5569,6 +6211,9 @@
       <c r="I226" t="n">
         <v>0.01212857142857143</v>
       </c>
+      <c r="J226" t="n">
+        <v>0.5496444444444444</v>
+      </c>
     </row>
     <row r="227">
       <c r="A227" s="1" t="n">
@@ -5592,6 +6237,9 @@
       <c r="I227" t="n">
         <v>0.01584</v>
       </c>
+      <c r="J227" t="n">
+        <v>0.5828166666666666</v>
+      </c>
     </row>
     <row r="228">
       <c r="A228" s="1" t="n">
@@ -5615,6 +6263,9 @@
       <c r="I228" t="n">
         <v>0.0123</v>
       </c>
+      <c r="J228" t="n">
+        <v>0.5203636363636363</v>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="1" t="n">
@@ -5638,6 +6289,9 @@
       <c r="I229" t="n">
         <v>0.0112</v>
       </c>
+      <c r="J229" t="n">
+        <v>0.564888888888889</v>
+      </c>
     </row>
     <row r="230">
       <c r="A230" s="1" t="n">
@@ -5661,6 +6315,9 @@
       <c r="I230" t="n">
         <v>0.01463333333333333</v>
       </c>
+      <c r="J230" t="n">
+        <v>0.5632777777777778</v>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="1" t="n">
@@ -5684,6 +6341,9 @@
       <c r="I231" t="n">
         <v>0.01574</v>
       </c>
+      <c r="J231" t="n">
+        <v>0.5177875000000001</v>
+      </c>
     </row>
     <row r="232">
       <c r="A232" s="1" t="n">
@@ -5707,6 +6367,9 @@
       <c r="I232" t="n">
         <v>0.01185</v>
       </c>
+      <c r="J232" t="n">
+        <v>0.5377307692307692</v>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="1" t="n">
@@ -5730,6 +6393,9 @@
       <c r="I233" t="n">
         <v>0.01116666666666667</v>
       </c>
+      <c r="J233" t="n">
+        <v>0.5020625000000001</v>
+      </c>
     </row>
     <row r="234">
       <c r="A234" s="1" t="n">
@@ -5753,6 +6419,9 @@
       <c r="I234" t="n">
         <v>0.01193333333333333</v>
       </c>
+      <c r="J234" t="n">
+        <v>0.6765333333333333</v>
+      </c>
     </row>
     <row r="235">
       <c r="A235" s="1" t="n">
@@ -5776,6 +6445,9 @@
       <c r="I235" t="n">
         <v>0.01456666666666667</v>
       </c>
+      <c r="J235" t="n">
+        <v>0.5295375</v>
+      </c>
     </row>
     <row r="236">
       <c r="A236" s="1" t="n">
@@ -5799,6 +6471,9 @@
       <c r="I236" t="n">
         <v>0.009285714285714286</v>
       </c>
+      <c r="J236" t="n">
+        <v>0.4566909090909091</v>
+      </c>
     </row>
     <row r="237">
       <c r="A237" s="1" t="n">
@@ -5822,6 +6497,9 @@
       <c r="I237" t="n">
         <v>0.0114</v>
       </c>
+      <c r="J237" t="n">
+        <v>0.3461</v>
+      </c>
     </row>
     <row r="238">
       <c r="A238" s="1" t="n">
@@ -5845,6 +6523,9 @@
       <c r="I238" t="n">
         <v>0.01131428571428571</v>
       </c>
+      <c r="J238" t="n">
+        <v>0.6089545454545454</v>
+      </c>
     </row>
     <row r="239">
       <c r="A239" s="1" t="n">
@@ -5868,6 +6549,9 @@
       <c r="I239" t="n">
         <v>0.0132</v>
       </c>
+      <c r="J239" t="n">
+        <v>0.5529818181818181</v>
+      </c>
     </row>
     <row r="240">
       <c r="A240" s="1" t="n">
@@ -5891,6 +6575,9 @@
       <c r="I240" t="n">
         <v>0.01398</v>
       </c>
+      <c r="J240" t="n">
+        <v>0.5207799999999999</v>
+      </c>
     </row>
     <row r="241">
       <c r="A241" s="1" t="n">
@@ -5914,6 +6601,9 @@
       <c r="I241" t="n">
         <v>0.00485</v>
       </c>
+      <c r="J241" t="n">
+        <v>0.5360666666666666</v>
+      </c>
     </row>
     <row r="242">
       <c r="A242" s="1" t="n">
@@ -5937,6 +6627,9 @@
       <c r="I242" t="n">
         <v>0.011225</v>
       </c>
+      <c r="J242" t="n">
+        <v>0.50887</v>
+      </c>
     </row>
     <row r="243">
       <c r="A243" s="1" t="n">
@@ -5960,6 +6653,9 @@
       <c r="I243" t="n">
         <v>0.009550000000000001</v>
       </c>
+      <c r="J243" t="n">
+        <v>0.4766727272727273</v>
+      </c>
     </row>
     <row r="244">
       <c r="A244" s="1" t="n">
@@ -5983,6 +6679,9 @@
       <c r="I244" t="n">
         <v>0.01535</v>
       </c>
+      <c r="J244" t="n">
+        <v>0.6740777777777778</v>
+      </c>
     </row>
     <row r="245">
       <c r="A245" s="1" t="n">
@@ -6006,6 +6705,9 @@
       <c r="I245" t="n">
         <v>0.01466666666666667</v>
       </c>
+      <c r="J245" t="n">
+        <v>0.5428363636363636</v>
+      </c>
     </row>
     <row r="246">
       <c r="A246" s="1" t="n">
@@ -6029,6 +6731,9 @@
       <c r="I246" t="n">
         <v>0.013525</v>
       </c>
+      <c r="J246" t="n">
+        <v>0.4670285714285715</v>
+      </c>
     </row>
     <row r="247">
       <c r="A247" s="1" t="n">
@@ -6052,6 +6757,9 @@
       <c r="I247" t="n">
         <v>0.01741666666666667</v>
       </c>
+      <c r="J247" t="n">
+        <v>0.4177</v>
+      </c>
     </row>
     <row r="248">
       <c r="A248" s="1" t="n">
@@ -6075,6 +6783,9 @@
       <c r="I248" t="n">
         <v>0.01104285714285714</v>
       </c>
+      <c r="J248" t="n">
+        <v>0.4193727272727273</v>
+      </c>
     </row>
     <row r="249">
       <c r="A249" s="1" t="n">
@@ -6098,6 +6809,9 @@
       <c r="I249" t="n">
         <v>0.0127375</v>
       </c>
+      <c r="J249" t="n">
+        <v>0.3126111111111111</v>
+      </c>
     </row>
     <row r="250">
       <c r="A250" s="1" t="n">
@@ -6121,6 +6835,9 @@
       <c r="I250" t="n">
         <v>0.0139</v>
       </c>
+      <c r="J250" t="n">
+        <v>0.52541</v>
+      </c>
     </row>
     <row r="251">
       <c r="A251" s="1" t="n">
@@ -6144,6 +6861,9 @@
       <c r="I251" t="n">
         <v>0.0115125</v>
       </c>
+      <c r="J251" t="n">
+        <v>0.62101</v>
+      </c>
     </row>
     <row r="252">
       <c r="A252" s="1" t="n">
@@ -6167,6 +6887,9 @@
       <c r="I252" t="n">
         <v>0.01378</v>
       </c>
+      <c r="J252" t="n">
+        <v>0.47405</v>
+      </c>
     </row>
     <row r="253">
       <c r="A253" s="1" t="n">
@@ -6190,6 +6913,9 @@
       <c r="I253" t="n">
         <v>0.008075000000000001</v>
       </c>
+      <c r="J253" t="n">
+        <v>0.2976124999999999</v>
+      </c>
     </row>
     <row r="254">
       <c r="A254" s="1" t="n">
@@ -6213,6 +6939,9 @@
       <c r="I254" t="n">
         <v>0.01317142857142857</v>
       </c>
+      <c r="J254" t="n">
+        <v>0.5305636363636363</v>
+      </c>
     </row>
     <row r="255">
       <c r="A255" s="1" t="n">
@@ -6236,6 +6965,9 @@
       <c r="I255" t="n">
         <v>0.0109</v>
       </c>
+      <c r="J255" t="n">
+        <v>0.453675</v>
+      </c>
     </row>
     <row r="256">
       <c r="A256" s="1" t="n">
@@ -6259,6 +6991,9 @@
       <c r="I256" t="n">
         <v>0.01064285714285714</v>
       </c>
+      <c r="J256" t="n">
+        <v>0.5264</v>
+      </c>
     </row>
     <row r="257">
       <c r="A257" s="1" t="n">
@@ -6282,6 +7017,9 @@
       <c r="I257" t="n">
         <v>0.0134</v>
       </c>
+      <c r="J257" t="n">
+        <v>0.5061099999999999</v>
+      </c>
     </row>
     <row r="258">
       <c r="A258" s="1" t="n">
@@ -6305,6 +7043,9 @@
       <c r="I258" t="n">
         <v>0.01263333333333333</v>
       </c>
+      <c r="J258" t="n">
+        <v>0.5704727272727272</v>
+      </c>
     </row>
     <row r="259">
       <c r="A259" s="1" t="n">
@@ -6328,6 +7069,9 @@
       <c r="I259" t="n">
         <v>0.01704285714285714</v>
       </c>
+      <c r="J259" t="n">
+        <v>0.4940125</v>
+      </c>
     </row>
     <row r="260">
       <c r="A260" s="1" t="n">
@@ -6351,6 +7095,9 @@
       <c r="I260" t="n">
         <v>0.01583333333333333</v>
       </c>
+      <c r="J260" t="n">
+        <v>0.49337</v>
+      </c>
     </row>
     <row r="261">
       <c r="A261" s="1" t="n">
@@ -6374,6 +7121,9 @@
       <c r="I261" t="n">
         <v>0.008433333333333334</v>
       </c>
+      <c r="J261" t="n">
+        <v>0.4787125</v>
+      </c>
     </row>
     <row r="262">
       <c r="A262" s="1" t="n">
@@ -6397,6 +7147,9 @@
       <c r="I262" t="n">
         <v>0.01156</v>
       </c>
+      <c r="J262" t="n">
+        <v>0.5332166666666667</v>
+      </c>
     </row>
     <row r="263">
       <c r="A263" s="1" t="n">
@@ -6420,6 +7173,9 @@
       <c r="I263" t="n">
         <v>0.0126875</v>
       </c>
+      <c r="J263" t="n">
+        <v>0.4821777777777778</v>
+      </c>
     </row>
     <row r="264">
       <c r="A264" s="1" t="n">
@@ -6443,6 +7199,9 @@
       <c r="I264" t="n">
         <v>0.01032857142857143</v>
       </c>
+      <c r="J264" t="n">
+        <v>0.2785666666666666</v>
+      </c>
     </row>
     <row r="265">
       <c r="A265" s="1" t="n">
@@ -6466,6 +7225,9 @@
       <c r="I265" t="n">
         <v>0.01536666666666667</v>
       </c>
+      <c r="J265" t="n">
+        <v>0.37362</v>
+      </c>
     </row>
     <row r="266">
       <c r="A266" s="1" t="n">
@@ -6489,6 +7251,9 @@
       <c r="I266" t="n">
         <v>0.01271666666666667</v>
       </c>
+      <c r="J266" t="n">
+        <v>0.5777333333333333</v>
+      </c>
     </row>
     <row r="267">
       <c r="A267" s="1" t="n">
@@ -6512,6 +7277,9 @@
       <c r="I267" t="n">
         <v>0.009600000000000001</v>
       </c>
+      <c r="J267" t="n">
+        <v>0.4187555555555555</v>
+      </c>
     </row>
     <row r="268">
       <c r="A268" s="1" t="n">
@@ -6535,6 +7303,9 @@
       <c r="I268" t="n">
         <v>0.008925000000000001</v>
       </c>
+      <c r="J268" t="n">
+        <v>0.4432923076923077</v>
+      </c>
     </row>
     <row r="269">
       <c r="A269" s="1" t="n">
@@ -6558,6 +7329,9 @@
       <c r="I269" t="n">
         <v>0.0111</v>
       </c>
+      <c r="J269" t="n">
+        <v>0.3992545454545455</v>
+      </c>
     </row>
     <row r="270">
       <c r="A270" s="1" t="n">
@@ -6581,6 +7355,9 @@
       <c r="I270" t="n">
         <v>0.015</v>
       </c>
+      <c r="J270" t="n">
+        <v>0.53024</v>
+      </c>
     </row>
     <row r="271">
       <c r="A271" s="1" t="n">
@@ -6604,6 +7381,9 @@
       <c r="I271" t="n">
         <v>0.0132</v>
       </c>
+      <c r="J271" t="n">
+        <v>0.35245</v>
+      </c>
     </row>
     <row r="272">
       <c r="A272" s="1" t="n">
@@ -6627,6 +7407,9 @@
       <c r="I272" t="n">
         <v>0.009800000000000001</v>
       </c>
+      <c r="J272" t="n">
+        <v>0.5364099999999999</v>
+      </c>
     </row>
     <row r="273">
       <c r="A273" s="1" t="n">
@@ -6650,6 +7433,9 @@
       <c r="I273" t="n">
         <v>0.01216</v>
       </c>
+      <c r="J273" t="n">
+        <v>0.49046</v>
+      </c>
     </row>
     <row r="274">
       <c r="A274" s="1" t="n">
@@ -6673,6 +7459,9 @@
       <c r="I274" t="n">
         <v>0.00855</v>
       </c>
+      <c r="J274" t="n">
+        <v>0.5271454545454546</v>
+      </c>
     </row>
     <row r="275">
       <c r="A275" s="1" t="n">
@@ -6696,6 +7485,9 @@
       <c r="I275" t="n">
         <v>0.0118</v>
       </c>
+      <c r="J275" t="n">
+        <v>0.6258583333333333</v>
+      </c>
     </row>
     <row r="276">
       <c r="A276" s="1" t="n">
@@ -6719,6 +7511,9 @@
       <c r="I276" t="n">
         <v>0.009800000000000001</v>
       </c>
+      <c r="J276" t="n">
+        <v>0.5662900000000001</v>
+      </c>
     </row>
     <row r="277">
       <c r="A277" s="1" t="n">
@@ -6742,6 +7537,9 @@
       <c r="I277" t="n">
         <v>0.01072</v>
       </c>
+      <c r="J277" t="n">
+        <v>0.5481333333333334</v>
+      </c>
     </row>
     <row r="278">
       <c r="A278" s="1" t="n">
@@ -6765,6 +7563,9 @@
       <c r="I278" t="n">
         <v>0.0097</v>
       </c>
+      <c r="J278" t="n">
+        <v>0.6872499999999999</v>
+      </c>
     </row>
     <row r="279">
       <c r="A279" s="1" t="n">
@@ -6788,6 +7589,9 @@
       <c r="I279" t="n">
         <v>0.00992</v>
       </c>
+      <c r="J279" t="n">
+        <v>0.38228</v>
+      </c>
     </row>
     <row r="280">
       <c r="A280" s="1" t="n">
@@ -6811,6 +7615,9 @@
       <c r="I280" t="n">
         <v>0.007571428571428571</v>
       </c>
+      <c r="J280" t="n">
+        <v>0.5379111111111111</v>
+      </c>
     </row>
     <row r="281">
       <c r="A281" s="1" t="n">
@@ -6834,6 +7641,9 @@
       <c r="I281" t="n">
         <v>0.008585714285714285</v>
       </c>
+      <c r="J281" t="n">
+        <v>0.3585</v>
+      </c>
     </row>
     <row r="282">
       <c r="A282" s="1" t="n">
@@ -6857,6 +7667,9 @@
       <c r="I282" t="n">
         <v>0.012675</v>
       </c>
+      <c r="J282" t="n">
+        <v>0.46475</v>
+      </c>
     </row>
     <row r="283">
       <c r="A283" s="1" t="n">
@@ -6880,6 +7693,9 @@
       <c r="I283" t="n">
         <v>0.009524999999999999</v>
       </c>
+      <c r="J283" t="n">
+        <v>0.5285444444444445</v>
+      </c>
     </row>
     <row r="284">
       <c r="A284" s="1" t="n">
@@ -6903,6 +7719,9 @@
       <c r="I284" t="n">
         <v>0.00856</v>
       </c>
+      <c r="J284" t="n">
+        <v>0.6937299999999998</v>
+      </c>
     </row>
     <row r="285">
       <c r="A285" s="1" t="n">
@@ -6926,6 +7745,9 @@
       <c r="I285" t="n">
         <v>0.008714285714285714</v>
       </c>
+      <c r="J285" t="n">
+        <v>0.619257142857143</v>
+      </c>
     </row>
     <row r="286">
       <c r="A286" s="1" t="n">
@@ -6949,6 +7771,9 @@
       <c r="I286" t="n">
         <v>0.0126</v>
       </c>
+      <c r="J286" t="n">
+        <v>0.4541099999999999</v>
+      </c>
     </row>
     <row r="287">
       <c r="A287" s="1" t="n">
@@ -6972,6 +7797,9 @@
       <c r="I287" t="n">
         <v>0.009650000000000001</v>
       </c>
+      <c r="J287" t="n">
+        <v>0.36542</v>
+      </c>
     </row>
     <row r="288">
       <c r="A288" s="1" t="n">
@@ -6995,6 +7823,9 @@
       <c r="I288" t="n">
         <v>0.007875</v>
       </c>
+      <c r="J288" t="n">
+        <v>0.4118777777777777</v>
+      </c>
     </row>
     <row r="289">
       <c r="A289" s="1" t="n">
@@ -7018,6 +7849,9 @@
       <c r="I289" t="n">
         <v>0.009479999999999999</v>
       </c>
+      <c r="J289" t="n">
+        <v>0.4954363636363638</v>
+      </c>
     </row>
     <row r="290">
       <c r="A290" s="1" t="n">
@@ -7041,6 +7875,9 @@
       <c r="I290" t="n">
         <v>0.009766666666666667</v>
       </c>
+      <c r="J290" t="n">
+        <v>0.5547111111111112</v>
+      </c>
     </row>
     <row r="291">
       <c r="A291" s="1" t="n">
@@ -7064,6 +7901,9 @@
       <c r="I291" t="n">
         <v>0.01</v>
       </c>
+      <c r="J291" t="n">
+        <v>0.4500666666666667</v>
+      </c>
     </row>
     <row r="292">
       <c r="A292" s="1" t="n">
@@ -7087,6 +7927,9 @@
       <c r="I292" t="n">
         <v>0.01084285714285714</v>
       </c>
+      <c r="J292" t="n">
+        <v>0.4856444444444444</v>
+      </c>
     </row>
     <row r="293">
       <c r="A293" s="1" t="n">
@@ -7110,6 +7953,9 @@
       <c r="I293" t="n">
         <v>0.01038333333333333</v>
       </c>
+      <c r="J293" t="n">
+        <v>0.5432083333333333</v>
+      </c>
     </row>
     <row r="294">
       <c r="A294" s="1" t="n">
@@ -7133,6 +7979,9 @@
       <c r="I294" t="n">
         <v>0.009942857142857142</v>
       </c>
+      <c r="J294" t="n">
+        <v>0.4857363636363636</v>
+      </c>
     </row>
     <row r="295">
       <c r="A295" s="1" t="n">
@@ -7156,6 +8005,9 @@
       <c r="I295" t="n">
         <v>0.004549999999999999</v>
       </c>
+      <c r="J295" t="n">
+        <v>0.43847</v>
+      </c>
     </row>
     <row r="296">
       <c r="A296" s="1" t="n">
@@ -7179,6 +8031,9 @@
       <c r="I296" t="n">
         <v>0.01044444444444444</v>
       </c>
+      <c r="J296" t="n">
+        <v>0.5291</v>
+      </c>
     </row>
     <row r="297">
       <c r="A297" s="1" t="n">
@@ -7202,6 +8057,9 @@
       <c r="I297" t="n">
         <v>0.01418571428571429</v>
       </c>
+      <c r="J297" t="n">
+        <v>0.5162</v>
+      </c>
     </row>
     <row r="298">
       <c r="A298" s="1" t="n">
@@ -7225,6 +8083,9 @@
       <c r="I298" t="n">
         <v>0.0051</v>
       </c>
+      <c r="J298" t="n">
+        <v>0.5041545454545454</v>
+      </c>
     </row>
     <row r="299">
       <c r="A299" s="1" t="n">
@@ -7248,6 +8109,9 @@
       <c r="I299" t="n">
         <v>0.0095625</v>
       </c>
+      <c r="J299" t="n">
+        <v>0.401623076923077</v>
+      </c>
     </row>
     <row r="300">
       <c r="A300" s="1" t="n">
@@ -7271,6 +8135,9 @@
       <c r="I300" t="n">
         <v>0.007180000000000001</v>
       </c>
+      <c r="J300" t="n">
+        <v>0.45561</v>
+      </c>
     </row>
     <row r="301">
       <c r="A301" s="1" t="n">
@@ -7294,6 +8161,9 @@
       <c r="I301" t="n">
         <v>0.01045</v>
       </c>
+      <c r="J301" t="n">
+        <v>0.3771777777777778</v>
+      </c>
     </row>
     <row r="302">
       <c r="A302" s="1" t="n">
@@ -7317,6 +8187,9 @@
       <c r="I302" t="n">
         <v>0.006874999999999999</v>
       </c>
+      <c r="J302" t="n">
+        <v>0.6104636363636364</v>
+      </c>
     </row>
     <row r="303">
       <c r="A303" s="1" t="n">
@@ -7340,6 +8213,9 @@
       <c r="I303" t="n">
         <v>0.009299999999999999</v>
       </c>
+      <c r="J303" t="n">
+        <v>0.4274909090909091</v>
+      </c>
     </row>
     <row r="304">
       <c r="A304" s="1" t="n">
@@ -7363,6 +8239,9 @@
       <c r="I304" t="n">
         <v>0.009949999999999999</v>
       </c>
+      <c r="J304" t="n">
+        <v>0.4839090909090908</v>
+      </c>
     </row>
     <row r="305">
       <c r="A305" s="1" t="n">
@@ -7386,6 +8265,9 @@
       <c r="I305" t="n">
         <v>0.007266666666666667</v>
       </c>
+      <c r="J305" t="n">
+        <v>0.6493749999999999</v>
+      </c>
     </row>
     <row r="306">
       <c r="A306" s="1" t="n">
@@ -7409,6 +8291,9 @@
       <c r="I306" t="n">
         <v>0.008333333333333333</v>
       </c>
+      <c r="J306" t="n">
+        <v>0.5018142857142857</v>
+      </c>
     </row>
     <row r="307">
       <c r="A307" s="1" t="n">
@@ -7432,6 +8317,9 @@
       <c r="I307" t="n">
         <v>0.00865</v>
       </c>
+      <c r="J307" t="n">
+        <v>0.4604571428571429</v>
+      </c>
     </row>
     <row r="308">
       <c r="A308" s="1" t="n">
@@ -7455,6 +8343,9 @@
       <c r="I308" t="n">
         <v>0.0086625</v>
       </c>
+      <c r="J308" t="n">
+        <v>0.4075545454545454</v>
+      </c>
     </row>
     <row r="309">
       <c r="A309" s="1" t="n">
@@ -7478,6 +8369,9 @@
       <c r="I309" t="n">
         <v>0.009639999999999999</v>
       </c>
+      <c r="J309" t="n">
+        <v>0.6233666666666667</v>
+      </c>
     </row>
     <row r="310">
       <c r="A310" s="1" t="n">
@@ -7501,6 +8395,9 @@
       <c r="I310" t="n">
         <v>0.01025</v>
       </c>
+      <c r="J310" t="n">
+        <v>0.5002555555555555</v>
+      </c>
     </row>
     <row r="311">
       <c r="A311" s="1" t="n">
@@ -7523,6 +8420,9 @@
       </c>
       <c r="I311" t="n">
         <v>0.01208333333333333</v>
+      </c>
+      <c r="J311" t="n">
+        <v>0.4580555555555555</v>
       </c>
     </row>
     <row r="314">
@@ -7571,6 +8471,9 @@
       <c r="I316" t="n">
         <v>0</v>
       </c>
+      <c r="J316" t="n">
+        <v>0.0002</v>
+      </c>
     </row>
     <row r="317">
       <c r="A317" s="1" t="n">
@@ -7594,6 +8497,9 @@
       <c r="I317" t="n">
         <v>0.0055</v>
       </c>
+      <c r="J317" t="n">
+        <v>0.0526</v>
+      </c>
     </row>
     <row r="318">
       <c r="A318" s="1" t="n">
@@ -7617,6 +8523,9 @@
       <c r="I318" t="n">
         <v>0.06370000000000001</v>
       </c>
+      <c r="J318" t="n">
+        <v>0.016</v>
+      </c>
     </row>
     <row r="319">
       <c r="A319" s="1" t="n">
@@ -7640,6 +8549,9 @@
       <c r="I319" t="n">
         <v>0.0674</v>
       </c>
+      <c r="J319" t="n">
+        <v>0.015</v>
+      </c>
     </row>
     <row r="320">
       <c r="A320" s="1" t="n">
@@ -7663,6 +8575,9 @@
       <c r="I320" t="n">
         <v>0.08749999999999999</v>
       </c>
+      <c r="J320" t="n">
+        <v>0.0237</v>
+      </c>
     </row>
     <row r="321">
       <c r="A321" s="1" t="n">
@@ -7686,6 +8601,9 @@
       <c r="I321" t="n">
         <v>0.06950000000000001</v>
       </c>
+      <c r="J321" t="n">
+        <v>0.0725</v>
+      </c>
     </row>
     <row r="322">
       <c r="A322" s="1" t="n">
@@ -7709,6 +8627,9 @@
       <c r="I322" t="n">
         <v>0.0859</v>
       </c>
+      <c r="J322" t="n">
+        <v>0.09470000000000001</v>
+      </c>
     </row>
     <row r="323">
       <c r="A323" s="1" t="n">
@@ -7732,6 +8653,9 @@
       <c r="I323" t="n">
         <v>0.0862</v>
       </c>
+      <c r="J323" t="n">
+        <v>0.0693</v>
+      </c>
     </row>
     <row r="324">
       <c r="A324" s="1" t="n">
@@ -7755,6 +8679,9 @@
       <c r="I324" t="n">
         <v>0.0916</v>
       </c>
+      <c r="J324" t="n">
+        <v>0.0493</v>
+      </c>
     </row>
     <row r="325">
       <c r="A325" s="1" t="n">
@@ -7778,6 +8705,9 @@
       <c r="I325" t="n">
         <v>0.09520000000000001</v>
       </c>
+      <c r="J325" t="n">
+        <v>0.0482</v>
+      </c>
     </row>
     <row r="326">
       <c r="A326" s="1" t="n">
@@ -7801,6 +8731,9 @@
       <c r="I326" t="n">
         <v>0.1071</v>
       </c>
+      <c r="J326" t="n">
+        <v>0.0401</v>
+      </c>
     </row>
     <row r="327">
       <c r="A327" s="1" t="n">
@@ -7824,6 +8757,9 @@
       <c r="I327" t="n">
         <v>0.1038</v>
       </c>
+      <c r="J327" t="n">
+        <v>0.0561</v>
+      </c>
     </row>
     <row r="328">
       <c r="A328" s="1" t="n">
@@ -7847,6 +8783,9 @@
       <c r="I328" t="n">
         <v>0.1017</v>
       </c>
+      <c r="J328" t="n">
+        <v>0.0392</v>
+      </c>
     </row>
     <row r="329">
       <c r="A329" s="1" t="n">
@@ -7870,6 +8809,9 @@
       <c r="I329" t="n">
         <v>0.1002</v>
       </c>
+      <c r="J329" t="n">
+        <v>0.0558</v>
+      </c>
     </row>
     <row r="330">
       <c r="A330" s="1" t="n">
@@ -7893,6 +8835,9 @@
       <c r="I330" t="n">
         <v>0.0965</v>
       </c>
+      <c r="J330" t="n">
+        <v>0.0553</v>
+      </c>
     </row>
     <row r="331">
       <c r="A331" s="1" t="n">
@@ -7916,6 +8861,9 @@
       <c r="I331" t="n">
         <v>0.0999</v>
       </c>
+      <c r="J331" t="n">
+        <v>0.0285</v>
+      </c>
     </row>
     <row r="332">
       <c r="A332" s="1" t="n">
@@ -7939,6 +8887,9 @@
       <c r="I332" t="n">
         <v>0.09660000000000001</v>
       </c>
+      <c r="J332" t="n">
+        <v>0.0508</v>
+      </c>
     </row>
     <row r="333">
       <c r="A333" s="1" t="n">
@@ -7962,6 +8913,9 @@
       <c r="I333" t="n">
         <v>0.0914</v>
       </c>
+      <c r="J333" t="n">
+        <v>0.07140000000000001</v>
+      </c>
     </row>
     <row r="334">
       <c r="A334" s="1" t="n">
@@ -7985,6 +8939,9 @@
       <c r="I334" t="n">
         <v>0.0992</v>
       </c>
+      <c r="J334" t="n">
+        <v>0.0398</v>
+      </c>
     </row>
     <row r="335">
       <c r="A335" s="1" t="n">
@@ -8008,6 +8965,9 @@
       <c r="I335" t="n">
         <v>0.09669999999999999</v>
       </c>
+      <c r="J335" t="n">
+        <v>0.0322</v>
+      </c>
     </row>
     <row r="336">
       <c r="A336" s="1" t="n">
@@ -8031,6 +8991,9 @@
       <c r="I336" t="n">
         <v>0.1047</v>
       </c>
+      <c r="J336" t="n">
+        <v>0.0294</v>
+      </c>
     </row>
     <row r="337">
       <c r="A337" s="1" t="n">
@@ -8054,6 +9017,9 @@
       <c r="I337" t="n">
         <v>0.1067</v>
       </c>
+      <c r="J337" t="n">
+        <v>0.0354</v>
+      </c>
     </row>
     <row r="338">
       <c r="A338" s="1" t="n">
@@ -8077,6 +9043,9 @@
       <c r="I338" t="n">
         <v>0.1036</v>
       </c>
+      <c r="J338" t="n">
+        <v>0.0385</v>
+      </c>
     </row>
     <row r="339">
       <c r="A339" s="1" t="n">
@@ -8100,6 +9069,9 @@
       <c r="I339" t="n">
         <v>0.1094</v>
       </c>
+      <c r="J339" t="n">
+        <v>0.0335</v>
+      </c>
     </row>
     <row r="340">
       <c r="A340" s="1" t="n">
@@ -8123,6 +9095,9 @@
       <c r="I340" t="n">
         <v>0.107</v>
       </c>
+      <c r="J340" t="n">
+        <v>0.0356</v>
+      </c>
     </row>
     <row r="341">
       <c r="A341" s="1" t="n">
@@ -8146,6 +9121,9 @@
       <c r="I341" t="n">
         <v>0.1023</v>
       </c>
+      <c r="J341" t="n">
+        <v>0.0394</v>
+      </c>
     </row>
     <row r="342">
       <c r="A342" s="1" t="n">
@@ -8169,6 +9147,9 @@
       <c r="I342" t="n">
         <v>0.1042</v>
       </c>
+      <c r="J342" t="n">
+        <v>0.042</v>
+      </c>
     </row>
     <row r="343">
       <c r="A343" s="1" t="n">
@@ -8192,6 +9173,9 @@
       <c r="I343" t="n">
         <v>0.1042</v>
       </c>
+      <c r="J343" t="n">
+        <v>0.0272</v>
+      </c>
     </row>
     <row r="344">
       <c r="A344" s="1" t="n">
@@ -8215,6 +9199,9 @@
       <c r="I344" t="n">
         <v>0.1025</v>
       </c>
+      <c r="J344" t="n">
+        <v>0.0345</v>
+      </c>
     </row>
     <row r="345">
       <c r="A345" s="1" t="n">
@@ -8238,6 +9225,9 @@
       <c r="I345" t="n">
         <v>0.1064</v>
       </c>
+      <c r="J345" t="n">
+        <v>0.0417</v>
+      </c>
     </row>
     <row r="346">
       <c r="A346" s="1" t="n">
@@ -8261,6 +9251,9 @@
       <c r="I346" t="n">
         <v>0.1087</v>
       </c>
+      <c r="J346" t="n">
+        <v>0.0375</v>
+      </c>
     </row>
     <row r="347">
       <c r="A347" s="1" t="n">
@@ -8284,6 +9277,9 @@
       <c r="I347" t="n">
         <v>0.1025</v>
       </c>
+      <c r="J347" t="n">
+        <v>0.0414</v>
+      </c>
     </row>
     <row r="348">
       <c r="A348" s="1" t="n">
@@ -8307,6 +9303,9 @@
       <c r="I348" t="n">
         <v>0.1041</v>
       </c>
+      <c r="J348" t="n">
+        <v>0.0342</v>
+      </c>
     </row>
     <row r="349">
       <c r="A349" s="1" t="n">
@@ -8330,6 +9329,9 @@
       <c r="I349" t="n">
         <v>0.1087</v>
       </c>
+      <c r="J349" t="n">
+        <v>0.0432</v>
+      </c>
     </row>
     <row r="350">
       <c r="A350" s="1" t="n">
@@ -8353,6 +9355,9 @@
       <c r="I350" t="n">
         <v>0.1041</v>
       </c>
+      <c r="J350" t="n">
+        <v>0.043</v>
+      </c>
     </row>
     <row r="351">
       <c r="A351" s="1" t="n">
@@ -8376,6 +9381,9 @@
       <c r="I351" t="n">
         <v>0.1029</v>
       </c>
+      <c r="J351" t="n">
+        <v>0.0282</v>
+      </c>
     </row>
     <row r="352">
       <c r="A352" s="1" t="n">
@@ -8399,6 +9407,9 @@
       <c r="I352" t="n">
         <v>0.1122</v>
       </c>
+      <c r="J352" t="n">
+        <v>0.0362</v>
+      </c>
     </row>
     <row r="353">
       <c r="A353" s="1" t="n">
@@ -8422,6 +9433,9 @@
       <c r="I353" t="n">
         <v>0.1004</v>
       </c>
+      <c r="J353" t="n">
+        <v>0.0443</v>
+      </c>
     </row>
     <row r="354">
       <c r="A354" s="1" t="n">
@@ -8445,6 +9459,9 @@
       <c r="I354" t="n">
         <v>0.1023</v>
       </c>
+      <c r="J354" t="n">
+        <v>0.0515</v>
+      </c>
     </row>
     <row r="355">
       <c r="A355" s="1" t="n">
@@ -8468,6 +9485,9 @@
       <c r="I355" t="n">
         <v>0.1064</v>
       </c>
+      <c r="J355" t="n">
+        <v>0.0294</v>
+      </c>
     </row>
     <row r="356">
       <c r="A356" s="1" t="n">
@@ -8491,6 +9511,9 @@
       <c r="I356" t="n">
         <v>0.107</v>
       </c>
+      <c r="J356" t="n">
+        <v>0.0305</v>
+      </c>
     </row>
     <row r="357">
       <c r="A357" s="1" t="n">
@@ -8514,6 +9537,9 @@
       <c r="I357" t="n">
         <v>0.1093</v>
       </c>
+      <c r="J357" t="n">
+        <v>0.0321</v>
+      </c>
     </row>
     <row r="358">
       <c r="A358" s="1" t="n">
@@ -8537,6 +9563,9 @@
       <c r="I358" t="n">
         <v>0.1152</v>
       </c>
+      <c r="J358" t="n">
+        <v>0.039</v>
+      </c>
     </row>
     <row r="359">
       <c r="A359" s="1" t="n">
@@ -8560,6 +9589,9 @@
       <c r="I359" t="n">
         <v>0.1091</v>
       </c>
+      <c r="J359" t="n">
+        <v>0.0455</v>
+      </c>
     </row>
     <row r="360">
       <c r="A360" s="1" t="n">
@@ -8583,6 +9615,9 @@
       <c r="I360" t="n">
         <v>0.1092</v>
       </c>
+      <c r="J360" t="n">
+        <v>0.032</v>
+      </c>
     </row>
     <row r="361">
       <c r="A361" s="1" t="n">
@@ -8606,6 +9641,9 @@
       <c r="I361" t="n">
         <v>0.1062</v>
       </c>
+      <c r="J361" t="n">
+        <v>0.0382</v>
+      </c>
     </row>
     <row r="362">
       <c r="A362" s="1" t="n">
@@ -8629,6 +9667,9 @@
       <c r="I362" t="n">
         <v>0.1017</v>
       </c>
+      <c r="J362" t="n">
+        <v>0.0446</v>
+      </c>
     </row>
     <row r="363">
       <c r="A363" s="1" t="n">
@@ -8652,6 +9693,9 @@
       <c r="I363" t="n">
         <v>0.109</v>
       </c>
+      <c r="J363" t="n">
+        <v>0.0287</v>
+      </c>
     </row>
     <row r="364">
       <c r="A364" s="1" t="n">
@@ -8675,6 +9719,9 @@
       <c r="I364" t="n">
         <v>0.1004</v>
       </c>
+      <c r="J364" t="n">
+        <v>0.0258</v>
+      </c>
     </row>
     <row r="365">
       <c r="A365" s="1" t="n">
@@ -8698,6 +9745,9 @@
       <c r="I365" t="n">
         <v>0.1137</v>
       </c>
+      <c r="J365" t="n">
+        <v>0.0368</v>
+      </c>
     </row>
     <row r="366">
       <c r="A366" s="1" t="n">
@@ -8721,6 +9771,9 @@
       <c r="I366" t="n">
         <v>0.1098</v>
       </c>
+      <c r="J366" t="n">
+        <v>0.0369</v>
+      </c>
     </row>
     <row r="367">
       <c r="A367" s="1" t="n">
@@ -8744,6 +9797,9 @@
       <c r="I367" t="n">
         <v>0.1129</v>
       </c>
+      <c r="J367" t="n">
+        <v>0.0319</v>
+      </c>
     </row>
     <row r="368">
       <c r="A368" s="1" t="n">
@@ -8767,6 +9823,9 @@
       <c r="I368" t="n">
         <v>0.1094</v>
       </c>
+      <c r="J368" t="n">
+        <v>0.0326</v>
+      </c>
     </row>
     <row r="369">
       <c r="A369" s="1" t="n">
@@ -8790,6 +9849,9 @@
       <c r="I369" t="n">
         <v>0.109</v>
       </c>
+      <c r="J369" t="n">
+        <v>0.0381</v>
+      </c>
     </row>
     <row r="370">
       <c r="A370" s="1" t="n">
@@ -8813,6 +9875,9 @@
       <c r="I370" t="n">
         <v>0.1095</v>
       </c>
+      <c r="J370" t="n">
+        <v>0.0297</v>
+      </c>
     </row>
     <row r="371">
       <c r="A371" s="1" t="n">
@@ -8836,6 +9901,9 @@
       <c r="I371" t="n">
         <v>0.1062</v>
       </c>
+      <c r="J371" t="n">
+        <v>0.027</v>
+      </c>
     </row>
     <row r="372">
       <c r="A372" s="1" t="n">
@@ -8859,6 +9927,9 @@
       <c r="I372" t="n">
         <v>0.1038</v>
       </c>
+      <c r="J372" t="n">
+        <v>0.0266</v>
+      </c>
     </row>
     <row r="373">
       <c r="A373" s="1" t="n">
@@ -8882,6 +9953,9 @@
       <c r="I373" t="n">
         <v>0.1075</v>
       </c>
+      <c r="J373" t="n">
+        <v>0.0433</v>
+      </c>
     </row>
     <row r="374">
       <c r="A374" s="1" t="n">
@@ -8905,6 +9979,9 @@
       <c r="I374" t="n">
         <v>0.1102</v>
       </c>
+      <c r="J374" t="n">
+        <v>0.0389</v>
+      </c>
     </row>
     <row r="375">
       <c r="A375" s="1" t="n">
@@ -8928,6 +10005,9 @@
       <c r="I375" t="n">
         <v>0.1013</v>
       </c>
+      <c r="J375" t="n">
+        <v>0.0271</v>
+      </c>
     </row>
     <row r="376">
       <c r="A376" s="1" t="n">
@@ -8951,6 +10031,9 @@
       <c r="I376" t="n">
         <v>0.105</v>
       </c>
+      <c r="J376" t="n">
+        <v>0.0274</v>
+      </c>
     </row>
     <row r="377">
       <c r="A377" s="1" t="n">
@@ -8974,6 +10057,9 @@
       <c r="I377" t="n">
         <v>0.1024</v>
       </c>
+      <c r="J377" t="n">
+        <v>0.032</v>
+      </c>
     </row>
     <row r="378">
       <c r="A378" s="1" t="n">
@@ -8997,6 +10083,9 @@
       <c r="I378" t="n">
         <v>0.1017</v>
       </c>
+      <c r="J378" t="n">
+        <v>0.0393</v>
+      </c>
     </row>
     <row r="379">
       <c r="A379" s="1" t="n">
@@ -9020,6 +10109,9 @@
       <c r="I379" t="n">
         <v>0.1078</v>
       </c>
+      <c r="J379" t="n">
+        <v>0.0429</v>
+      </c>
     </row>
     <row r="380">
       <c r="A380" s="1" t="n">
@@ -9043,6 +10135,9 @@
       <c r="I380" t="n">
         <v>0.1036</v>
       </c>
+      <c r="J380" t="n">
+        <v>0.0336</v>
+      </c>
     </row>
     <row r="381">
       <c r="A381" s="1" t="n">
@@ -9066,6 +10161,9 @@
       <c r="I381" t="n">
         <v>0.1055</v>
       </c>
+      <c r="J381" t="n">
+        <v>0.0257</v>
+      </c>
     </row>
     <row r="382">
       <c r="A382" s="1" t="n">
@@ -9089,6 +10187,9 @@
       <c r="I382" t="n">
         <v>0.1053</v>
       </c>
+      <c r="J382" t="n">
+        <v>0.0257</v>
+      </c>
     </row>
     <row r="383">
       <c r="A383" s="1" t="n">
@@ -9112,6 +10213,9 @@
       <c r="I383" t="n">
         <v>0.1031</v>
       </c>
+      <c r="J383" t="n">
+        <v>0.0262</v>
+      </c>
     </row>
     <row r="384">
       <c r="A384" s="1" t="n">
@@ -9135,6 +10239,9 @@
       <c r="I384" t="n">
         <v>0.1075</v>
       </c>
+      <c r="J384" t="n">
+        <v>0.0275</v>
+      </c>
     </row>
     <row r="385">
       <c r="A385" s="1" t="n">
@@ -9158,6 +10265,9 @@
       <c r="I385" t="n">
         <v>0.1096</v>
       </c>
+      <c r="J385" t="n">
+        <v>0.0242</v>
+      </c>
     </row>
     <row r="386">
       <c r="A386" s="1" t="n">
@@ -9181,6 +10291,9 @@
       <c r="I386" t="n">
         <v>0.1143</v>
       </c>
+      <c r="J386" t="n">
+        <v>0.028</v>
+      </c>
     </row>
     <row r="387">
       <c r="A387" s="1" t="n">
@@ -9204,6 +10317,9 @@
       <c r="I387" t="n">
         <v>0.1039</v>
       </c>
+      <c r="J387" t="n">
+        <v>0.0338</v>
+      </c>
     </row>
     <row r="388">
       <c r="A388" s="1" t="n">
@@ -9227,6 +10343,9 @@
       <c r="I388" t="n">
         <v>0.1091</v>
       </c>
+      <c r="J388" t="n">
+        <v>0.0229</v>
+      </c>
     </row>
     <row r="389">
       <c r="A389" s="1" t="n">
@@ -9250,6 +10369,9 @@
       <c r="I389" t="n">
         <v>0.1013</v>
       </c>
+      <c r="J389" t="n">
+        <v>0.0264</v>
+      </c>
     </row>
     <row r="390">
       <c r="A390" s="1" t="n">
@@ -9273,6 +10395,9 @@
       <c r="I390" t="n">
         <v>0.1079</v>
       </c>
+      <c r="J390" t="n">
+        <v>0.027</v>
+      </c>
     </row>
     <row r="391">
       <c r="A391" s="1" t="n">
@@ -9296,6 +10421,9 @@
       <c r="I391" t="n">
         <v>0.0989</v>
       </c>
+      <c r="J391" t="n">
+        <v>0.0313</v>
+      </c>
     </row>
     <row r="392">
       <c r="A392" s="1" t="n">
@@ -9319,6 +10447,9 @@
       <c r="I392" t="n">
         <v>0.1047</v>
       </c>
+      <c r="J392" t="n">
+        <v>0.0238</v>
+      </c>
     </row>
     <row r="393">
       <c r="A393" s="1" t="n">
@@ -9342,6 +10473,9 @@
       <c r="I393" t="n">
         <v>0.1025</v>
       </c>
+      <c r="J393" t="n">
+        <v>0.0217</v>
+      </c>
     </row>
     <row r="394">
       <c r="A394" s="1" t="n">
@@ -9365,6 +10499,9 @@
       <c r="I394" t="n">
         <v>0.1004</v>
       </c>
+      <c r="J394" t="n">
+        <v>0.0193</v>
+      </c>
     </row>
     <row r="395">
       <c r="A395" s="1" t="n">
@@ -9388,6 +10525,9 @@
       <c r="I395" t="n">
         <v>0.1001</v>
       </c>
+      <c r="J395" t="n">
+        <v>0.0251</v>
+      </c>
     </row>
     <row r="396">
       <c r="A396" s="1" t="n">
@@ -9411,6 +10551,9 @@
       <c r="I396" t="n">
         <v>0.109</v>
       </c>
+      <c r="J396" t="n">
+        <v>0.027</v>
+      </c>
     </row>
     <row r="397">
       <c r="A397" s="1" t="n">
@@ -9434,6 +10577,9 @@
       <c r="I397" t="n">
         <v>0.1085</v>
       </c>
+      <c r="J397" t="n">
+        <v>0.024</v>
+      </c>
     </row>
     <row r="398">
       <c r="A398" s="1" t="n">
@@ -9457,6 +10603,9 @@
       <c r="I398" t="n">
         <v>0.1079</v>
       </c>
+      <c r="J398" t="n">
+        <v>0.0319</v>
+      </c>
     </row>
     <row r="399">
       <c r="A399" s="1" t="n">
@@ -9480,6 +10629,9 @@
       <c r="I399" t="n">
         <v>0.1023</v>
       </c>
+      <c r="J399" t="n">
+        <v>0.0279</v>
+      </c>
     </row>
     <row r="400">
       <c r="A400" s="1" t="n">
@@ -9503,6 +10655,9 @@
       <c r="I400" t="n">
         <v>0.1054</v>
       </c>
+      <c r="J400" t="n">
+        <v>0.0276</v>
+      </c>
     </row>
     <row r="401">
       <c r="A401" s="1" t="n">
@@ -9526,6 +10681,9 @@
       <c r="I401" t="n">
         <v>0.1044</v>
       </c>
+      <c r="J401" t="n">
+        <v>0.0218</v>
+      </c>
     </row>
     <row r="402">
       <c r="A402" s="1" t="n">
@@ -9549,6 +10707,9 @@
       <c r="I402" t="n">
         <v>0.1009</v>
       </c>
+      <c r="J402" t="n">
+        <v>0.0215</v>
+      </c>
     </row>
     <row r="403">
       <c r="A403" s="1" t="n">
@@ -9572,6 +10733,9 @@
       <c r="I403" t="n">
         <v>0.109</v>
       </c>
+      <c r="J403" t="n">
+        <v>0.019</v>
+      </c>
     </row>
     <row r="404">
       <c r="A404" s="1" t="n">
@@ -9595,6 +10759,9 @@
       <c r="I404" t="n">
         <v>0.1049</v>
       </c>
+      <c r="J404" t="n">
+        <v>0.0241</v>
+      </c>
     </row>
     <row r="405">
       <c r="A405" s="1" t="n">
@@ -9618,6 +10785,9 @@
       <c r="I405" t="n">
         <v>0.1052</v>
       </c>
+      <c r="J405" t="n">
+        <v>0.0263</v>
+      </c>
     </row>
     <row r="406">
       <c r="A406" s="1" t="n">
@@ -9641,6 +10811,9 @@
       <c r="I406" t="n">
         <v>0.1057</v>
       </c>
+      <c r="J406" t="n">
+        <v>0.0262</v>
+      </c>
     </row>
     <row r="407">
       <c r="A407" s="1" t="n">
@@ -9664,6 +10837,9 @@
       <c r="I407" t="n">
         <v>0.1032</v>
       </c>
+      <c r="J407" t="n">
+        <v>0.0338</v>
+      </c>
     </row>
     <row r="408">
       <c r="A408" s="1" t="n">
@@ -9687,6 +10863,9 @@
       <c r="I408" t="n">
         <v>0.1052</v>
       </c>
+      <c r="J408" t="n">
+        <v>0.0286</v>
+      </c>
     </row>
     <row r="409">
       <c r="A409" s="1" t="n">
@@ -9710,6 +10889,9 @@
       <c r="I409" t="n">
         <v>0.1071</v>
       </c>
+      <c r="J409" t="n">
+        <v>0.0255</v>
+      </c>
     </row>
     <row r="410">
       <c r="A410" s="1" t="n">
@@ -9733,6 +10915,9 @@
       <c r="I410" t="n">
         <v>0.1138</v>
       </c>
+      <c r="J410" t="n">
+        <v>0.0225</v>
+      </c>
     </row>
     <row r="411">
       <c r="A411" s="1" t="n">
@@ -9756,6 +10941,9 @@
       <c r="I411" t="n">
         <v>0.1059</v>
       </c>
+      <c r="J411" t="n">
+        <v>0.0247</v>
+      </c>
     </row>
     <row r="412">
       <c r="A412" s="1" t="n">
@@ -9779,6 +10967,9 @@
       <c r="I412" t="n">
         <v>0.1004</v>
       </c>
+      <c r="J412" t="n">
+        <v>0.0217</v>
+      </c>
     </row>
     <row r="413">
       <c r="A413" s="1" t="n">
@@ -9802,6 +10993,9 @@
       <c r="I413" t="n">
         <v>0.1041</v>
       </c>
+      <c r="J413" t="n">
+        <v>0.028</v>
+      </c>
     </row>
     <row r="414">
       <c r="A414" s="1" t="n">
@@ -9825,6 +11019,9 @@
       <c r="I414" t="n">
         <v>0.1</v>
       </c>
+      <c r="J414" t="n">
+        <v>0.0238</v>
+      </c>
     </row>
     <row r="415">
       <c r="A415" s="1" t="n">
@@ -9847,6 +11044,9 @@
       </c>
       <c r="I415" t="n">
         <v>0.102</v>
+      </c>
+      <c r="J415" t="n">
+        <v>0.0239</v>
       </c>
     </row>
   </sheetData>

</xml_diff>